<commit_message>
V1.5 ||| rounted corners, relayouted ZB2, SAMTEC connectors now dnp
</commit_message>
<xml_diff>
--- a/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
+++ b/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ELSYS\repos\uz_mz_adapter\MicroZohmVorgabe\Project Outputs for uz_mz_adapter\Rev01\BOM_JLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ELSYS\repos\uz_mz_adapter\Breakout\Project Outputs for uz_mz_adapter\Rev01\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0AD5A47-D329-453F-A13D-89C462040122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{26938E98-289F-4FB4-967A-CF6DD0C3D0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-150" windowWidth="29040" windowHeight="15720" xr2:uid="{84F826CA-EEF6-4A08-AF30-6DE632F4FE4B}"/>
+    <workbookView xWindow="28680" yWindow="-150" windowWidth="29040" windowHeight="15720" xr2:uid="{BC8ACB1A-3968-418A-89BD-15C14699A550}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_uz_mz_adapter_Variant_V" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
   <si>
     <t>Name</t>
   </si>
@@ -249,24 +249,6 @@
   </si>
   <si>
     <t>C492401</t>
-  </si>
-  <si>
-    <t>IPL1-115-01-L-D-RA-K</t>
-  </si>
-  <si>
-    <t>X1-1, X2-1, X3-1, X4-1</t>
-  </si>
-  <si>
-    <t>IPL1-115-01-XX-D-RA</t>
-  </si>
-  <si>
-    <t>IPL1-120-01-L-D-RA-K</t>
-  </si>
-  <si>
-    <t>X1-2, X2-2, X3-2</t>
-  </si>
-  <si>
-    <t>IPL1-120-01-XX-D-RA</t>
   </si>
   <si>
     <t>ERM8-060-02.0-L-DV-TR</t>
@@ -367,7 +349,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -383,7 +365,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -698,14 +680,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9667C4A-0866-495A-B0AF-ECF9B1ECFC1B}">
-  <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6987F209-A6C9-4CF5-842B-AF2EAEBF805E}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" customWidth="1"/>
-    <col min="3" max="3" width="24.28515625" customWidth="1"/>
-    <col min="4" max="5" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" customWidth="1"/>
+    <col min="4" max="5" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1003,79 +985,49 @@
       <c r="C18" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D18" s="1"/>
+      <c r="D18" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="E18" s="2" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>77</v>
+        <v>45</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B21" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>86</v>
-      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
V1.6 ||| updated npn bjt
</commit_message>
<xml_diff>
--- a/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
+++ b/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ELSYS\repos\uz_mz_adapter\Breakout\Project Outputs for uz_mz_adapter\Rev01\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26938E98-289F-4FB4-967A-CF6DD0C3D0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{29F32A3C-E7CE-445E-BDFA-16A45C7BC7F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-150" windowWidth="29040" windowHeight="15720" xr2:uid="{BC8ACB1A-3968-418A-89BD-15C14699A550}"/>
+    <workbookView xWindow="6495" yWindow="2025" windowWidth="17280" windowHeight="11790" xr2:uid="{1FAD54A3-C93F-464A-A831-BA6A781BC3E1}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_uz_mz_adapter_Variant_V" sheetId="1" r:id="rId1"/>
@@ -140,13 +140,13 @@
     <t>C84269</t>
   </si>
   <si>
-    <t>19-213/Y2C-CQ2R2L/3T(CY)</t>
+    <t>150060YS75000</t>
   </si>
   <si>
     <t>D4</t>
   </si>
   <si>
-    <t>C72038</t>
+    <t>C6784997</t>
   </si>
   <si>
     <t>6339160-1</t>
@@ -161,16 +161,16 @@
     <t>C125076</t>
   </si>
   <si>
-    <t>BC846BLT3G</t>
+    <t>SBC846BLT3G</t>
   </si>
   <si>
     <t>Q1</t>
   </si>
   <si>
-    <t>SOT95P280X145-3N</t>
-  </si>
-  <si>
-    <t>C513271</t>
+    <t>SOT-23-3_ONSC</t>
+  </si>
+  <si>
+    <t>C896883</t>
   </si>
   <si>
     <t>4k3</t>
@@ -680,7 +680,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6987F209-A6C9-4CF5-842B-AF2EAEBF805E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D96362C4-E744-4821-AF49-4D97F954B0CC}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
V1.7 ||| cahnged gen components to actual c numbers
</commit_message>
<xml_diff>
--- a/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
+++ b/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ELSYS\repos\uz_mz_adapter\Breakout\Project Outputs for uz_mz_adapter\Rev01\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{29F32A3C-E7CE-445E-BDFA-16A45C7BC7F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7BE51FE-256F-4071-92AB-831CFA03945B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6495" yWindow="2025" windowWidth="17280" windowHeight="11790" xr2:uid="{1FAD54A3-C93F-464A-A831-BA6A781BC3E1}"/>
+    <workbookView xWindow="35640" yWindow="2340" windowWidth="17280" windowHeight="11790" xr2:uid="{B9FA3D30-A537-448F-A1A3-F5DC1E5DF32D}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_uz_mz_adapter_Variant_V" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="84">
   <si>
     <t>Name</t>
   </si>
@@ -95,19 +95,28 @@
     <t>C5</t>
   </si>
   <si>
+    <t>C_0603</t>
+  </si>
+  <si>
+    <t>C2177372</t>
+  </si>
+  <si>
+    <t>C0603C105K3RAC7411</t>
+  </si>
+  <si>
+    <t>10 u</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
     <t>C_0603_TE</t>
   </si>
   <si>
-    <t>UZgen_C_0603_1uF_16V_X7R</t>
-  </si>
-  <si>
-    <t>10 µF</t>
-  </si>
-  <si>
-    <t>C6</t>
-  </si>
-  <si>
-    <t>UZgen_C_0603_10uF_16V_X7R</t>
+    <t>C22367826</t>
+  </si>
+  <si>
+    <t>HGC0603R5106K350NTHJ</t>
   </si>
   <si>
     <t>150060BS84000</t>
@@ -341,9 +350,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -680,7 +688,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D96362C4-E744-4821-AF49-4D97F954B0CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{761B71D2-2D26-4D0C-BEF8-51F78D7B3110}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -690,340 +698,344 @@
     <col min="4" max="5" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="E4" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>22</v>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="A7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>26</v>
+      <c r="D7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>29</v>
+      <c r="A8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>32</v>
+      <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>35</v>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>39</v>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>47</v>
       </c>
+      <c r="C12" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>51</v>
+      <c r="D13" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="B14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>59</v>
       </c>
+      <c r="B15" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>64</v>
       </c>
+      <c r="C16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>65</v>
+      <c r="B17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>69</v>
+      <c r="B18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>73</v>
+      <c r="B19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="A20" s="1" t="s">
         <v>80</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V1.9 ||| updated RJ45 bc of availability
</commit_message>
<xml_diff>
--- a/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
+++ b/Breakout/Project Outputs for uz_mz_adapter/Rev01/BOM_JLC/BOM_JLC_uz_mz_adapter_Variant_V1_Rev01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ELSYS\repos\uz_mz_adapter\Breakout\Project Outputs for uz_mz_adapter\Rev01\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7BE51FE-256F-4071-92AB-831CFA03945B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2678FD5B-19E2-4FE5-941B-9CEAAC98FE97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35640" yWindow="2340" windowWidth="17280" windowHeight="11790" xr2:uid="{B9FA3D30-A537-448F-A1A3-F5DC1E5DF32D}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{D0DB9C1E-4B6E-4850-B1C4-C47A89220386}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_uz_mz_adapter_Variant_V" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="92">
   <si>
     <t>Name</t>
   </si>
@@ -158,16 +158,16 @@
     <t>C6784997</t>
   </si>
   <si>
-    <t>6339160-1</t>
+    <t>RJHSE-3381</t>
   </si>
   <si>
     <t>J1, J2, J3, J4, J5, J6, J7, J8</t>
   </si>
   <si>
-    <t>634008149821</t>
-  </si>
-  <si>
-    <t>C125076</t>
+    <t>RJ45-TH_RJHSE-3381</t>
+  </si>
+  <si>
+    <t>C599439</t>
   </si>
   <si>
     <t>SBC846BLT3G</t>
@@ -258,6 +258,30 @@
   </si>
   <si>
     <t>C492401</t>
+  </si>
+  <si>
+    <t>IPL1-115-01-L-D-K</t>
+  </si>
+  <si>
+    <t>X1-1, X2-1, X3-1, X4-1</t>
+  </si>
+  <si>
+    <t>IPL1-115-01-YYY-D-K</t>
+  </si>
+  <si>
+    <t>C17431809</t>
+  </si>
+  <si>
+    <t>IPL1-120-01-L-D-K</t>
+  </si>
+  <si>
+    <t>X1-2, X2-2, X3-2</t>
+  </si>
+  <si>
+    <t>SAMTEC_IPL1-120-01-X-D-K</t>
+  </si>
+  <si>
+    <t>C17429670</t>
   </si>
   <si>
     <t>ERM8-060-02.0-L-DV-TR</t>
@@ -688,8 +712,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{761B71D2-2D26-4D0C-BEF8-51F78D7B3110}">
-  <dimension ref="A1:E20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8710BB3F-0DC5-4B6E-9B7D-1E20B7D9FEC5}">
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
@@ -1029,13 +1053,47 @@
         <v>81</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>83</v>
+      <c r="D22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>